<commit_message>
Update DateBase/orders/Dang Nguyen 195_2026-8-8.xlsx
</commit_message>
<xml_diff>
--- a/DateBase/orders/Dang Nguyen 195_2026-8-8.xlsx
+++ b/DateBase/orders/Dang Nguyen 195_2026-8-8.xlsx
@@ -598,6 +598,9 @@
       <c r="C21" t="str">
         <v>803_烟花菊粉紫_undefined_undefined_1bunch</v>
       </c>
+      <c r="F21" t="str">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
@@ -656,7 +659,7 @@
         <v>0.00</v>
       </c>
       <c r="G2" t="str">
-        <v>0101010101010101010101020101510551050</v>
+        <v>0101010101010101010101020101510551055</v>
       </c>
     </row>
   </sheetData>

</xml_diff>